<commit_message>
Thiet ke trang luyen de v15
</commit_message>
<xml_diff>
--- a/ETS2023_Test1_Final_Architecture.xlsx
+++ b/ETS2023_Test1_Final_Architecture.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28035" windowHeight="11730" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28035" windowHeight="11730"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Info" sheetId="1" r:id="rId1"/>
@@ -2728,9 +2728,6 @@
     <t>P6_02</t>
   </si>
   <si>
-    <t>Gasgo Propane Tank Exchange&lt;br&gt;&lt;br&gt;You have chosen a safe and _______(135) way to obtain fuel for your stoves, grills, heaters, fireplaces, or other devices. Simply follow the directions _______(136).&lt;br&gt;&lt;br&gt;When your tank runs out of propane, take it to our store and leave it on one of the clearly marked green shelves outside the store. _______(137). Then, pay the cashier inside the store for a fresh tank of propane. Next, the cashier or another staff member will accompany you to the outdoor exchange area. The staff person will give you a full tank to take home and provide help if you have multiple tanks to carry. Follow the instructions on the tank to connect it to your device.&lt;br&gt;&lt;br&gt;Be sure to visit us again when you need a _______(138).</t>
-  </si>
-  <si>
     <t>You have chosen a safe and _______ way to obtain fuel...</t>
   </si>
   <si>
@@ -2803,9 +2800,6 @@
     <t>P6_03</t>
   </si>
   <si>
-    <t>To: Technicarn Enterprises Customers&lt;br&gt;From: Technicarn Enterprises Customer Service&lt;br&gt;Date: 10 September&lt;br&gt;Subject: Serving You&lt;br&gt;&lt;br&gt;Dear Valued Customer:&lt;br&gt;We want your _______(139) with Technicarn Enterprises to be easy and enjoyable. To that end, we are pleased to announce our newly designed Web site, with enhanced customer-friendly features.&lt;br&gt;&lt;br&gt;Our new Web site provides answers to your questions 24 hours a day, every day of the year. On our home page, you can get information about system setup, or you can troubleshoot by visiting _______(140) the Internet Issues or TV and Streaming Issues pages. _______(141), you can find detailed information concerning account management, access, billing, and payment.&lt;br&gt;&lt;br&gt;Please explore the new Web site at your earliest convenience: www.technicarnenterprises.com. _______(142). As always, thank you for allowing us to serve you.</t>
-  </si>
-  <si>
     <t>We want your _______ with Technicarn Enterprises to be easy and enjoyable.</t>
   </si>
   <si>
@@ -2878,9 +2872,6 @@
     <t>P6_04</t>
   </si>
   <si>
-    <t>Garner City Transport Cares About the Environment&lt;br&gt;&lt;br&gt;Beginning May 1, the sale and use of paper tickets and transit passes will be _______(143) on all Garner City Transport bus and subway lines. This change applies to single-ride tickets _______(144) to weekly and monthly passes. Eliminating paper benefits the environment and leads to less litter.&lt;br&gt;&lt;br&gt;Riders can download the free Garner City Transport app. With the app, they can add money their accounts, purchase tickets, plan _______(145), and track arrival and departure times.&lt;br&gt;&lt;br&gt;Alternatively, passengers can purchase a rechargeable transit card at any station. Value can be added to the card via the Garner City Transport Web site at www.garnercitytransport.org. _______(146).</t>
-  </si>
-  <si>
     <t>Beginning May 1, the sale and use of paper tickets and transit passes will be _______ on all Garner City Transport bus and subway lines.</t>
   </si>
   <si>
@@ -2953,9 +2944,6 @@
     <t>P7_01</t>
   </si>
   <si>
-    <t>Harbis Stationery Store Clearance Sale&lt;br&gt;Prices indicated are for in-store purchases only.&lt;br&gt;500 Pinstone Street / SHEFFIELD / S12HN&lt;br&gt;&lt;br&gt;Seasonal items&lt;br&gt;- Box of ten preprinted seasonal cards (25% off): £ 8.99&lt;br&gt;- Box of five customizable seasonal cards or invitations (50% off): £ 11.99&lt;br&gt;&lt;br&gt;All school supplies 10% off&lt;br&gt;- Box of 24 pens: £ 1.79&lt;br&gt;- Desk lamp: £ 19.99&lt;br&gt;- Wireless mouse: £ 17.99&lt;br&gt;- Backpack: £ 29.99&lt;br&gt;&lt;br&gt;Visit Harbis Stationery at www.harbisstationery.uk</t>
-  </si>
-  <si>
     <t>What is indicated about Harbis Stationery Store?</t>
   </si>
   <si>
@@ -2995,9 +2983,6 @@
     <t>P7_02</t>
   </si>
   <si>
-    <t>To: Wenbin Peng &lt;wpeng@chenconstruction.com&gt;&lt;br&gt;From: Toshi Auto Group &lt;cs@toshiautogroup.com&gt;&lt;br&gt;Date: February 26&lt;br&gt;Subject: Your leased vehicle&lt;br&gt;&lt;br&gt;Dear Mr. Peng:&lt;br&gt;As you know, Toshi Auto Group handles all the service needs for cars leased by employees of Chen Construction. According to our records, you took possession of your leased car on March 1 of last year. Your car is now due for its required annual service and maintenance check. To book your appointment, please call us at (215) 555-0109 or visit us online at www.toshiautogroup.com/serviceappointments.&lt;br&gt;&lt;br&gt;Sincerely,&lt;br&gt;Toshi Auto Group Customer Service</t>
-  </si>
-  <si>
     <t>What is the purpose of the e-mail?</t>
   </si>
   <si>
@@ -3037,9 +3022,6 @@
     <t>P7_03</t>
   </si>
   <si>
-    <t>LONDON (2 February)-On Thursday, Tillford Press announced the launch of its new imprint, Tillford Exalt. This new line will feature books promoting healthy lifestyles, memoirs with uplifting messages, and volumes that provide guidance for special occasions such as birthdays and weddings...&lt;br&gt;Already contracted to write memoirs are the award-winning actress Alexia Leoz, London-based conductor and composer Seung-Hyun Bae, and celebrity cook Lain Lai. Ms. Lai's story of her life and career will be the first to be launched. It is set for release in December.&lt;br&gt;...Tillford Press is based in Manchester. It has offices in New York, Toronto, and Sydney, but its publications are sold throughout the world.</t>
-  </si>
-  <si>
     <t>What is the main purpose of the article?</t>
   </si>
   <si>
@@ -3094,9 +3076,6 @@
     <t>P7_04</t>
   </si>
   <si>
-    <t>Greg Skagen (8:58 A.M.) Hi, Brenda. I'm here in the warehouse. All of my trainees have arrived, but I noticed the power door at Loading Dock B is acting up.&lt;br&gt;Brenda Sadauskas (8:59 A.M.) Again?&lt;br&gt;Greg Skagen (8:59 A.M.) When I push the button to open it, it raises all the way up but then drops back down to the closed position after about 30 seconds.&lt;br&gt;Brenda Sadauskas (9:00 A.M.) I'll come down with the maintenance technicians. Why don't you bring your trainees to my area? You can teach them how to create shipping labels and then have them pack and label this morning's shipments.&lt;br&gt;Greg Skagen (9:02 A.M.) Yes, that works.&lt;br&gt;Brenda Sadauskas (9:03 A.M.) Thanks. Then you could show them the loading dock operations in the afternoon.</t>
-  </si>
-  <si>
     <t>What problem does Mr. Skagen mention?</t>
   </si>
   <si>
@@ -3136,9 +3115,6 @@
     <t>P7_05</t>
   </si>
   <si>
-    <t>SERVICE REQUEST FORM&lt;br&gt;Requester Name: Elenora Deckow&lt;br&gt;Requester Office: Room 718&lt;br&gt;Service Location: Room 500&lt;br&gt;Service Type: Repair&lt;br&gt;Description of Request:&lt;br&gt;There is a problem with the television audio. When I played an online video, the image was fine, but I could not hear anything. I checked all the settings, and I was able to hear the same video on other televisions with no problem. I'm supposed to deliver a product demonstration for a client in room 500 next Monday, so I would greatly appreciate it if the issue can be fixed by this Friday.</t>
-  </si>
-  <si>
     <t>Why was the form submitted?</t>
   </si>
   <si>
@@ -3178,9 +3154,6 @@
     <t>P7_06</t>
   </si>
   <si>
-    <t>Ella Glatt (11:34 A.M.) Hi. I know this is a busy day, but I wanted to know whether anyone from the finance team could come to the marketing meeting.&lt;br&gt;Stef Goldberg (11:35 A.M.) Hi, Ella. I wish I could, but it starts at 2:00. I need to be at a different meeting at 2:30.&lt;br&gt;Ella Glatt (11:36 A.M.) Oh, right. I forgot you were going to the executive board meeting.&lt;br&gt;Daniel Seidal (11:36 A.M.) I'm also supposed to go to the 2:30 meeting. Is it essential that one of us attend the marketing meeting?&lt;br&gt;Ella Glatt (11:37 A.M.) Well, it would be helpful to have someone from the finance department there, at least for 15 minutes or so.&lt;br&gt;Bill Iverman (11:38 A.M.) The quarterly reports just came in, and Daniel, Stef, and I need to review them by the end of the day.&lt;br&gt;Daniel Seidal (11:41 A.M.) That's true! But I could come from 2:00 to 2:15. That's all I can commit to.&lt;br&gt;Ella Glatt (11:43 A.M.) Sounds great. We just need one of you to clarify a few quick points about the budget for the next advertising campaign.</t>
-  </si>
-  <si>
     <t>At what time will the executive board meeting begin?</t>
   </si>
   <si>
@@ -3256,9 +3229,6 @@
     <t>P7_07</t>
   </si>
   <si>
-    <t>To: amal.abboud@bunzifoundation.org&lt;br&gt;From: maria_mcfarland@myemail.com&lt;br&gt;Date: Thursday, August 22&lt;br&gt;Subject: Project Coordinator Position&lt;br&gt;Attachment: résumé_m.mcfarland.pdf&lt;br&gt;&lt;br&gt;Dear Mr. Abboud,&lt;br&gt;My friend Josiah Wilkins told me that you are seeking a project coordinator for your company. I have a degree in business administration and am attaching my résumé as I think I am an excellent fit for your needs. As you will see, I have experience using several cloud-based project-management programs.&lt;br&gt;&lt;br&gt;My current role as project coordinator for an international engineering firm... has afforded me ample experience managing teams, schedules, and budgets. While I enjoy the kind of work I do, it has become clear to me that I need motivation from a strong mission. The goal of your company to create sustainable housing projects is something that I strongly support and would be delighted to work on.&lt;br&gt;&lt;br&gt;Through my work and volunteer activities, I have spent many months abroad in various countries throughout Asia and the Middle East. This seems particularly relevant to mention, as I am comfortable leading geographically and culturally diverse teams.</t>
-  </si>
-  <si>
     <t>What does Ms. McFarland mention about Mr. Wilkins?</t>
   </si>
   <si>
@@ -3334,9 +3304,6 @@
     <t>P7_08</t>
   </si>
   <si>
-    <t>About Our Company&lt;br&gt;Trexdale Supply specializes in designing, producing, and installing furniture for all types of scientific laboratories. We provide a range of fully assembled cabinets, workstations, benches, and more... Our lab furniture is available in a wide variety of sizes.&lt;br&gt;&lt;br&gt;Our business offers products as well as design-consulting services. For start-up labs, we have a team of consulting specialists available to evaluate your facility's specific needs and assist you in arranging your space... Recently, for example, we were chosen by a major producer of biofuels to provide expert help in changing the layout of a research laboratory to maximize available space.&lt;br&gt;&lt;br&gt;Please visit the "Lab Planning" section of this Web site if you are interested in learning more... There, you can fill out an interest form to contact one of our consultants.</t>
-  </si>
-  <si>
     <t>What does Trexdale Supply make?</t>
   </si>
   <si>
@@ -3394,9 +3361,6 @@
     <t>P7_09</t>
   </si>
   <si>
-    <t>PRODUCT DEMONSTRATORS NEEDED!&lt;br&gt;Are you outgoing and enthusiastic?- [1]. Do you enjoy talking to all types of people? Put your personality and communication skills to work! - [2] -. BBD Staffing is seeking to hire in-store product demonstrators to promote our clients' merchandise to shoppers. - [3]. As a member of our team, you will demonstrate a wide range of small kitchen appliances and tools in grocery stores and other retail venues.&lt;br&gt;&lt;br&gt;For some products, you will be required to prepare simple recipes. You will also need to answer shoppers' questions. Thus, it is essential that you can become familiar with clients' products and provide key information to consumers. Because many of the demonstrations require working with food, candidates must have a Professional Food Handler certificate. - [4] -.&lt;br&gt;&lt;br&gt;To apply, upload a video of no more than one minute in length telling us why you would be a successful product demonstrator at www.bbdstaffing.com/applications.</t>
-  </si>
-  <si>
     <t>What work experience would best qualify a candidate for the position?</t>
   </si>
   <si>
@@ -3454,9 +3418,6 @@
     <t>P7_10</t>
   </si>
   <si>
-    <t>Gorman Unveils Newest Smartphone Model&lt;br&gt;&lt;br&gt;LONDON (20 April)-Gorman Mobile unveiled its newest smartphone to an eager reception at the annual Technobrit Conference. The Pro Phone 4, which includes 512 GB of storage, a 7-inch screen display, and an optional stylus pen, will hit the shelves on 11 June. Unlike its predecessor the Pro Phone 3-it features a larger screen, an ultrawide camera lens, and 8K-resolution filming capability.&lt;br&gt;&lt;br&gt;[1]. The £999 starting price is £100 more than that of the previous model. Add-ons, such as the stylus pen, protective case, and wireless headphones, cost an additional £39, £59, and £79, respectively. Gorman Product Manager Ian Hill doesn't believe the price increase will dissuade customers.&lt;br&gt;&lt;br&gt;[2] - "The Pro Phone 4 is a game changer in terms of its picture quality and sleek design." said Hill. "Improvements were based on direct customer feedback..."&lt;br&gt;&lt;br&gt;[3] -. One similarity that the Pro Phone 4 has with previous models is the charger...&lt;br&gt;&lt;br&gt;"We want to afford our customers the ability to reuse elements of the other Gorman devices they've already purchased," said Hill. "Why add to the overload of cables already in circulation?" - [4]-</t>
-  </si>
-  <si>
     <t>What is the purpose of the article?</t>
   </si>
   <si>
@@ -3520,9 +3481,6 @@
     <t>P7_11</t>
   </si>
   <si>
-    <t>WORK ORDER: 7549&lt;br&gt;Requester: Xi, Gina&lt;br&gt;Date Entered: Wednesday, 9 April&lt;br&gt;Type: Technology end-user request&lt;br&gt;Technician Assigned: Arnold, Sam&lt;br&gt;Description: Is it possible to remove the new layers of security on my voice mail in the new phone system? I really don't want to use a password, and I certainly don't want to change it every month. I don't need a high degree of security because my work is not confidential. If someone else gained access to my messages, it wouldn't do much harm.&lt;br&gt;&lt;br&gt;E-mail&lt;br&gt;To: Gina Xi&lt;br&gt;From: Sam Arnold&lt;br&gt;Subject: Tech support request 7549&lt;br&gt;Hello, Ms. Xi. This is in reference to your work order 7549 related to the new phone system... I understand that you do not feel that a high degree of security is needed for your voice-mail settings, but the new system does require you to have a password to retrieve your voice mail. However, company policy allows me to change the settings for employees who do not work with confidential material. I can update the security settings so that you do not have to reset the password on a regular basis... If you still feel comfortable with that level of risk, let me know, and I will change the settings so that your password never expires.</t>
-  </si>
-  <si>
     <t>What does Ms. Xi's request indicate about the company?</t>
   </si>
   <si>
@@ -3616,9 +3574,6 @@
     <t>P7_12</t>
   </si>
   <si>
-    <t>E-mail&lt;br&gt;To: Linda Hanshu&lt;br&gt;From: Cliff Merson&lt;br&gt;Subject: Lighting Issue&lt;br&gt;I want to check on the issue we discussed about lighting in the latest chapter of Titan Adventure. In past versions of the game, getting the reflections and lighting in green and blue areas correct has been a particular challenge... As the new release, Neptune's Voyage, is primarily an underwater adventure, addressing this problem is crucial. You said you would take charge of this, and I hope to hear that you have found a solution... The team was hoping to have one last rendering of the lighting for the game by October 10...&lt;br&gt;&lt;br&gt;Review of Titan Adventure: Neptune's Voyage&lt;br&gt;By Leo Weber, April 1&lt;br&gt;This new installment of Titan Adventure will surprise and delight both new players and old aficionados... This newest version also corrects the green and blue image rendering that was sometimes a problem in earlier installments of Titan Adventure. Neptune's Voyage launches May 5 on Rimerko Clutch and FS5. It is available in English, Korean, Japanese, French, and Spanish.</t>
-  </si>
-  <si>
     <t>In the e-mail, what is suggested about Mr. Merson?</t>
   </si>
   <si>
@@ -3712,9 +3667,6 @@
     <t>P7_13</t>
   </si>
   <si>
-    <t>Wonder Ridge Radio Broadcast Schedule&lt;br&gt;Noon-4 P.M. AFTERNOON JAZZ. Music from traditional jazz to jazz fusion. Host: Malachi Mzee&lt;br&gt;4 P.M.-7 P.M. FOLK FRENZY. Folk music from around the world. Host: Penny Ariza&lt;br&gt;7 P.M.-10 P.M. JOSIE'S JOINT. Modern sounds selected by our station's own music director. Host: Josie Jones&lt;br&gt;&lt;br&gt;E-mail: To the folks at Wonder Ridge Radio:&lt;br&gt;As I was driving last week... Suddenly, my car was filled with a song that I hadn't heard in many years. It was traditional music from France, where my grandmother was born... I never expected to hear it on the radio here in Wonder Ridge. Thanks for this experience... Pierre Fabre&lt;br&gt;&lt;br&gt;Job Opening: Programming Assistant&lt;br&gt;Responsibilities: Conducting background research on interviewees. Keeping up-to-date on news... Updating the station's Web site and program host biography pages. Using scheduling software to update the broadcast schedule...</t>
-  </si>
-  <si>
     <t>According to the schedule, who is Ms. Jones?</t>
   </si>
   <si>
@@ -3805,9 +3757,6 @@
     <t>P7_14</t>
   </si>
   <si>
-    <t>Instructions for Requesting Records&lt;br&gt;1. Create an account in the Records Center Web portal. Currently, all requests must be made through the portal.&lt;br&gt;2. Use the drop-down menu to locate the department from which you are seeking information and submit your request. You will receive a confirmation e-mail with a reference number.&lt;br&gt;3. The department staff will locate the requested records and contact you when they are available... If you prefer to pick them up in person, you must make an appointment with the department staff.&lt;br&gt;&lt;br&gt;E-Mail Message&lt;br&gt;To: Joo-Hee Park &lt;jhpark@coa.net&gt;&lt;br&gt;From: Keith Brandenberg &lt;kbrandenberg@mailcurrent.com&gt;&lt;br&gt;Dear Ms. Park... I have a question about the fee. Apparently, I am being charged $300 for my documents. I do not understand why the fee is so high... I am only requesting two maps of the city's underground pipelines, which will inform our firm's current work advising the city on wastewater management.&lt;br&gt;&lt;br&gt;Sign: City of Abilene Administrative Building&lt;br&gt;First-Floor Directory:&lt;br&gt;IT Services - Room 100&lt;br&gt;Parks and Recreation - Room 101&lt;br&gt;Transportation - Room 102&lt;br&gt;Wastewater - Room 103</t>
-  </si>
-  <si>
     <t>What do the instructions indicate about records requests?</t>
   </si>
   <si>
@@ -3901,9 +3850,6 @@
     <t>P7_15</t>
   </si>
   <si>
-    <t>Review: Famous Actor, First Book&lt;br&gt;Fans of Simon Eklund will be delighted with his autobiography, The Theatre Lights Dimmed, the first book he has written in his storied career as an actor. It provides wonderful insight into his career, starting with his first roles in cinema in his native Sweden, moving into his work in France and Italy, and finishing with his recent theatre work in the U.K... -Uma Joshi&lt;br&gt;&lt;br&gt;E-mail 1&lt;br&gt;To: Edith Hocking | From: Uma Joshi | Date: 2 March&lt;br&gt;Thank you for agreeing to arrange an interview with Mr. Eklund for me. I think this will be a great follow-up to my recent piece. In a helpful coincidence, I will be visiting his home country next month to address a journalists' convention. I am the featured speaker and will discuss the benefits of diversity in journalism.&lt;br&gt;&lt;br&gt;E-mail 2&lt;br&gt;To: Uma Joshi | From: Maria Cazalla&lt;br&gt;We are all very excited about your interview next month with Mr. Eklund. He enjoys all your writing for Top News U.K.-the news stories, interviews, and, of course, your recent article about The Theatre Lights Dimmed! I just wanted to finalize a few details with you. We have arranged transportation for you from your hotel to Mr. Eklund's house and then back to the hotel. Please let me know how many people there will be in your group, because Mr. Eklund would like you all to stay for lunch.</t>
-  </si>
-  <si>
     <t>What does the review mention about Mr. Eklund?</t>
   </si>
   <si>
@@ -3994,9 +3940,6 @@
     <t>Giải thích: Maria viết trong email thứ 2 rằng: Ông Eklund thích tất cả bài viết của bà, và tất nhiên là CẢ bài báo/review gần đây về cuốn tự truyện của ông ấy ('your recent article about The Theatre Lights Dimmed!') -&gt; Ông ấy hài lòng với bài review của Joshi.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Audio/main/ETS2023_Test1_Full.mp3</t>
-  </si>
-  <si>
     <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/main/p1_01.png</t>
   </si>
   <si>
@@ -4031,6 +3974,63 @@
   </si>
   <si>
     <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_131.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_135.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_139.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_143.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_147.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_149.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_151.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_154.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_156.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_158.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_162.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_166.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_169.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_172.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_176(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_176(2).png </t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_181(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_181(2).png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(3).png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(3).png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(3).png</t>
+  </si>
+  <si>
+    <t>https://github.com/bangvang1105-tech/Audio-Test-1-ETS-2023/raw/refs/heads/main/Test%201%20ETS%202023.mp3</t>
   </si>
 </sst>
 </file>
@@ -4492,7 +4492,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>1324</v>
+        <v>1336</v>
       </c>
       <c r="D2" s="2">
         <v>120</v>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="8" t="s">
-        <v>1325</v>
+        <v>1306</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="9" t="s">
-        <v>1326</v>
+        <v>1307</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="8" t="s">
-        <v>1327</v>
+        <v>1308</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="9" t="s">
-        <v>1328</v>
+        <v>1309</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="8" t="s">
-        <v>1329</v>
+        <v>1310</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="9" t="s">
-        <v>1330</v>
+        <v>1311</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="D64" s="5"/>
       <c r="E64" s="8" t="s">
-        <v>1331</v>
+        <v>1312</v>
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5" t="s">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="9" t="s">
-        <v>1332</v>
+        <v>1313</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="D70" s="5"/>
       <c r="E70" s="8" t="s">
-        <v>1333</v>
+        <v>1314</v>
       </c>
       <c r="F70" s="5"/>
       <c r="G70" s="5" t="s">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="9" t="s">
-        <v>1334</v>
+        <v>1315</v>
       </c>
       <c r="F97" s="6"/>
       <c r="G97" s="6" t="s">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="D100" s="5"/>
       <c r="E100" s="8" t="s">
-        <v>1335</v>
+        <v>1316</v>
       </c>
       <c r="F100" s="5"/>
       <c r="G100" s="5" t="s">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="D132" s="5"/>
       <c r="E132" s="8" t="s">
-        <v>1336</v>
+        <v>1317</v>
       </c>
       <c r="F132" s="5"/>
       <c r="G132" s="5" t="s">
@@ -9263,7 +9263,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="136" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>135</v>
       </c>
@@ -9274,30 +9274,30 @@
         <v>901</v>
       </c>
       <c r="D136" s="5"/>
-      <c r="E136" s="5"/>
-      <c r="F136" s="5" t="s">
+      <c r="E136" s="8" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5" t="s">
         <v>902</v>
       </c>
-      <c r="G136" s="5" t="s">
+      <c r="H136" s="5" t="s">
         <v>903</v>
       </c>
-      <c r="H136" s="5" t="s">
+      <c r="I136" s="5" t="s">
         <v>904</v>
       </c>
-      <c r="I136" s="5" t="s">
+      <c r="J136" s="5" t="s">
         <v>905</v>
       </c>
-      <c r="J136" s="5" t="s">
+      <c r="K136" s="5" t="s">
         <v>906</v>
-      </c>
-      <c r="K136" s="5" t="s">
-        <v>907</v>
       </c>
       <c r="L136" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M136" s="5" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.25">
@@ -9314,25 +9314,25 @@
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
       <c r="G137" s="6" t="s">
+        <v>908</v>
+      </c>
+      <c r="H137" s="6" t="s">
         <v>909</v>
       </c>
-      <c r="H137" s="6" t="s">
+      <c r="I137" s="6" t="s">
         <v>910</v>
       </c>
-      <c r="I137" s="6" t="s">
+      <c r="J137" s="6" t="s">
         <v>911</v>
       </c>
-      <c r="J137" s="6" t="s">
+      <c r="K137" s="6" t="s">
         <v>912</v>
-      </c>
-      <c r="K137" s="6" t="s">
-        <v>913</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M137" s="6" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="138" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -9352,22 +9352,22 @@
         <v>883</v>
       </c>
       <c r="H138" s="5" t="s">
+        <v>914</v>
+      </c>
+      <c r="I138" s="5" t="s">
         <v>915</v>
       </c>
-      <c r="I138" s="5" t="s">
+      <c r="J138" s="5" t="s">
         <v>916</v>
       </c>
-      <c r="J138" s="5" t="s">
+      <c r="K138" s="5" t="s">
         <v>917</v>
-      </c>
-      <c r="K138" s="5" t="s">
-        <v>918</v>
       </c>
       <c r="L138" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M138" s="5" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="139" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -9384,28 +9384,28 @@
       <c r="E139" s="6"/>
       <c r="F139" s="6"/>
       <c r="G139" s="6" t="s">
+        <v>919</v>
+      </c>
+      <c r="H139" s="6" t="s">
         <v>920</v>
       </c>
-      <c r="H139" s="6" t="s">
+      <c r="I139" s="6" t="s">
         <v>921</v>
       </c>
-      <c r="I139" s="6" t="s">
+      <c r="J139" s="6" t="s">
         <v>922</v>
       </c>
-      <c r="J139" s="6" t="s">
+      <c r="K139" s="6" t="s">
         <v>923</v>
-      </c>
-      <c r="K139" s="6" t="s">
-        <v>924</v>
       </c>
       <c r="L139" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M139" s="6" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="140" spans="1:13" ht="180" x14ac:dyDescent="0.25">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="140" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>139</v>
       </c>
@@ -9413,33 +9413,33 @@
         <v>6</v>
       </c>
       <c r="C140" s="4" t="s">
+        <v>925</v>
+      </c>
+      <c r="D140" s="5"/>
+      <c r="E140" s="8" t="s">
+        <v>1319</v>
+      </c>
+      <c r="F140" s="5"/>
+      <c r="G140" s="5" t="s">
         <v>926</v>
       </c>
-      <c r="D140" s="5"/>
-      <c r="E140" s="5"/>
-      <c r="F140" s="5" t="s">
+      <c r="H140" s="5" t="s">
         <v>927</v>
       </c>
-      <c r="G140" s="5" t="s">
+      <c r="I140" s="5" t="s">
         <v>928</v>
       </c>
-      <c r="H140" s="5" t="s">
+      <c r="J140" s="5" t="s">
         <v>929</v>
       </c>
-      <c r="I140" s="5" t="s">
+      <c r="K140" s="5" t="s">
         <v>930</v>
-      </c>
-      <c r="J140" s="5" t="s">
-        <v>931</v>
-      </c>
-      <c r="K140" s="5" t="s">
-        <v>932</v>
       </c>
       <c r="L140" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M140" s="5" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
     </row>
     <row r="141" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -9450,31 +9450,31 @@
         <v>6</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
       <c r="F141" s="6"/>
       <c r="G141" s="6" t="s">
+        <v>932</v>
+      </c>
+      <c r="H141" s="6" t="s">
+        <v>933</v>
+      </c>
+      <c r="I141" s="6" t="s">
         <v>934</v>
       </c>
-      <c r="H141" s="6" t="s">
+      <c r="J141" s="6" t="s">
         <v>935</v>
       </c>
-      <c r="I141" s="6" t="s">
+      <c r="K141" s="6" t="s">
         <v>936</v>
-      </c>
-      <c r="J141" s="6" t="s">
-        <v>937</v>
-      </c>
-      <c r="K141" s="6" t="s">
-        <v>938</v>
       </c>
       <c r="L141" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M141" s="6" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
     </row>
     <row r="142" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -9485,31 +9485,31 @@
         <v>6</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D142" s="5"/>
       <c r="E142" s="5"/>
       <c r="F142" s="5"/>
       <c r="G142" s="5" t="s">
+        <v>938</v>
+      </c>
+      <c r="H142" s="5" t="s">
+        <v>939</v>
+      </c>
+      <c r="I142" s="5" t="s">
         <v>940</v>
       </c>
-      <c r="H142" s="5" t="s">
+      <c r="J142" s="5" t="s">
         <v>941</v>
       </c>
-      <c r="I142" s="5" t="s">
+      <c r="K142" s="5" t="s">
         <v>942</v>
-      </c>
-      <c r="J142" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="K142" s="5" t="s">
-        <v>944</v>
       </c>
       <c r="L142" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M142" s="5" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
     </row>
     <row r="143" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -9520,7 +9520,7 @@
         <v>6</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
@@ -9529,25 +9529,25 @@
         <v>883</v>
       </c>
       <c r="H143" s="6" t="s">
+        <v>944</v>
+      </c>
+      <c r="I143" s="6" t="s">
+        <v>945</v>
+      </c>
+      <c r="J143" s="6" t="s">
         <v>946</v>
       </c>
-      <c r="I143" s="6" t="s">
+      <c r="K143" s="6" t="s">
         <v>947</v>
-      </c>
-      <c r="J143" s="6" t="s">
-        <v>948</v>
-      </c>
-      <c r="K143" s="6" t="s">
-        <v>949</v>
       </c>
       <c r="L143" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M143" s="6" t="s">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="144" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="144" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>143</v>
       </c>
@@ -9555,33 +9555,33 @@
         <v>6</v>
       </c>
       <c r="C144" s="4" t="s">
+        <v>949</v>
+      </c>
+      <c r="D144" s="5"/>
+      <c r="E144" s="8" t="s">
+        <v>1320</v>
+      </c>
+      <c r="F144" s="5"/>
+      <c r="G144" s="5" t="s">
+        <v>950</v>
+      </c>
+      <c r="H144" s="5" t="s">
         <v>951</v>
       </c>
-      <c r="D144" s="5"/>
-      <c r="E144" s="5"/>
-      <c r="F144" s="5" t="s">
+      <c r="I144" s="5" t="s">
         <v>952</v>
       </c>
-      <c r="G144" s="5" t="s">
+      <c r="J144" s="5" t="s">
         <v>953</v>
       </c>
-      <c r="H144" s="5" t="s">
+      <c r="K144" s="5" t="s">
         <v>954</v>
-      </c>
-      <c r="I144" s="5" t="s">
-        <v>955</v>
-      </c>
-      <c r="J144" s="5" t="s">
-        <v>956</v>
-      </c>
-      <c r="K144" s="5" t="s">
-        <v>957</v>
       </c>
       <c r="L144" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M144" s="5" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
     </row>
     <row r="145" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -9592,31 +9592,31 @@
         <v>6</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
       <c r="G145" s="6" t="s">
+        <v>956</v>
+      </c>
+      <c r="H145" s="6" t="s">
+        <v>957</v>
+      </c>
+      <c r="I145" s="6" t="s">
+        <v>958</v>
+      </c>
+      <c r="J145" s="6" t="s">
         <v>959</v>
       </c>
-      <c r="H145" s="6" t="s">
+      <c r="K145" s="6" t="s">
         <v>960</v>
-      </c>
-      <c r="I145" s="6" t="s">
-        <v>961</v>
-      </c>
-      <c r="J145" s="6" t="s">
-        <v>962</v>
-      </c>
-      <c r="K145" s="6" t="s">
-        <v>963</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M145" s="6" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
     </row>
     <row r="146" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -9627,31 +9627,31 @@
         <v>6</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>
       <c r="F146" s="5"/>
       <c r="G146" s="5" t="s">
+        <v>962</v>
+      </c>
+      <c r="H146" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="I146" s="5" t="s">
+        <v>964</v>
+      </c>
+      <c r="J146" s="5" t="s">
         <v>965</v>
       </c>
-      <c r="H146" s="5" t="s">
+      <c r="K146" s="5" t="s">
         <v>966</v>
-      </c>
-      <c r="I146" s="5" t="s">
-        <v>967</v>
-      </c>
-      <c r="J146" s="5" t="s">
-        <v>968</v>
-      </c>
-      <c r="K146" s="5" t="s">
-        <v>969</v>
       </c>
       <c r="L146" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M146" s="5" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
     </row>
     <row r="147" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -9662,7 +9662,7 @@
         <v>6</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
@@ -9671,25 +9671,25 @@
         <v>883</v>
       </c>
       <c r="H147" s="6" t="s">
+        <v>968</v>
+      </c>
+      <c r="I147" s="6" t="s">
+        <v>969</v>
+      </c>
+      <c r="J147" s="6" t="s">
+        <v>970</v>
+      </c>
+      <c r="K147" s="6" t="s">
         <v>971</v>
-      </c>
-      <c r="I147" s="6" t="s">
-        <v>972</v>
-      </c>
-      <c r="J147" s="6" t="s">
-        <v>973</v>
-      </c>
-      <c r="K147" s="6" t="s">
-        <v>974</v>
       </c>
       <c r="L147" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M147" s="6" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="148" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="148" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>147</v>
       </c>
@@ -9697,33 +9697,33 @@
         <v>7</v>
       </c>
       <c r="C148" s="4" t="s">
+        <v>973</v>
+      </c>
+      <c r="D148" s="5"/>
+      <c r="E148" s="8" t="s">
+        <v>1321</v>
+      </c>
+      <c r="F148" s="5"/>
+      <c r="G148" s="5" t="s">
+        <v>974</v>
+      </c>
+      <c r="H148" s="5" t="s">
+        <v>975</v>
+      </c>
+      <c r="I148" s="5" t="s">
         <v>976</v>
       </c>
-      <c r="D148" s="5"/>
-      <c r="E148" s="5"/>
-      <c r="F148" s="5" t="s">
+      <c r="J148" s="5" t="s">
         <v>977</v>
       </c>
-      <c r="G148" s="5" t="s">
+      <c r="K148" s="5" t="s">
         <v>978</v>
-      </c>
-      <c r="H148" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="I148" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="J148" s="5" t="s">
-        <v>981</v>
-      </c>
-      <c r="K148" s="5" t="s">
-        <v>982</v>
       </c>
       <c r="L148" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M148" s="5" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
     </row>
     <row r="149" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -9734,34 +9734,34 @@
         <v>7</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
       <c r="G149" s="6" t="s">
+        <v>980</v>
+      </c>
+      <c r="H149" s="6" t="s">
+        <v>981</v>
+      </c>
+      <c r="I149" s="6" t="s">
+        <v>982</v>
+      </c>
+      <c r="J149" s="6" t="s">
+        <v>983</v>
+      </c>
+      <c r="K149" s="6" t="s">
         <v>984</v>
-      </c>
-      <c r="H149" s="6" t="s">
-        <v>985</v>
-      </c>
-      <c r="I149" s="6" t="s">
-        <v>986</v>
-      </c>
-      <c r="J149" s="6" t="s">
-        <v>987</v>
-      </c>
-      <c r="K149" s="6" t="s">
-        <v>988</v>
       </c>
       <c r="L149" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M149" s="6" t="s">
-        <v>989</v>
-      </c>
-    </row>
-    <row r="150" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="150" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>149</v>
       </c>
@@ -9769,33 +9769,33 @@
         <v>7</v>
       </c>
       <c r="C150" s="4" t="s">
+        <v>986</v>
+      </c>
+      <c r="D150" s="5"/>
+      <c r="E150" s="8" t="s">
+        <v>1322</v>
+      </c>
+      <c r="F150" s="5"/>
+      <c r="G150" s="5" t="s">
+        <v>987</v>
+      </c>
+      <c r="H150" s="5" t="s">
+        <v>988</v>
+      </c>
+      <c r="I150" s="5" t="s">
+        <v>989</v>
+      </c>
+      <c r="J150" s="5" t="s">
         <v>990</v>
       </c>
-      <c r="D150" s="5"/>
-      <c r="E150" s="5"/>
-      <c r="F150" s="5" t="s">
+      <c r="K150" s="5" t="s">
         <v>991</v>
-      </c>
-      <c r="G150" s="5" t="s">
-        <v>992</v>
-      </c>
-      <c r="H150" s="5" t="s">
-        <v>993</v>
-      </c>
-      <c r="I150" s="5" t="s">
-        <v>994</v>
-      </c>
-      <c r="J150" s="5" t="s">
-        <v>995</v>
-      </c>
-      <c r="K150" s="5" t="s">
-        <v>996</v>
       </c>
       <c r="L150" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M150" s="5" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="151" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -9806,34 +9806,34 @@
         <v>7</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
       <c r="G151" s="6" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
       <c r="H151" s="6" t="s">
-        <v>999</v>
+        <v>994</v>
       </c>
       <c r="I151" s="6" t="s">
-        <v>1000</v>
+        <v>995</v>
       </c>
       <c r="J151" s="6" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="K151" s="6" t="s">
-        <v>1002</v>
+        <v>997</v>
       </c>
       <c r="L151" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M151" s="6" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="152" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="152" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>151</v>
       </c>
@@ -9841,33 +9841,33 @@
         <v>7</v>
       </c>
       <c r="C152" s="4" t="s">
+        <v>999</v>
+      </c>
+      <c r="D152" s="5"/>
+      <c r="E152" s="8" t="s">
+        <v>1323</v>
+      </c>
+      <c r="F152" s="5"/>
+      <c r="G152" s="5" t="s">
+        <v>1000</v>
+      </c>
+      <c r="H152" s="5" t="s">
+        <v>1001</v>
+      </c>
+      <c r="I152" s="5" t="s">
+        <v>1002</v>
+      </c>
+      <c r="J152" s="5" t="s">
+        <v>1003</v>
+      </c>
+      <c r="K152" s="5" t="s">
         <v>1004</v>
-      </c>
-      <c r="D152" s="5"/>
-      <c r="E152" s="5"/>
-      <c r="F152" s="5" t="s">
-        <v>1005</v>
-      </c>
-      <c r="G152" s="5" t="s">
-        <v>1006</v>
-      </c>
-      <c r="H152" s="5" t="s">
-        <v>1007</v>
-      </c>
-      <c r="I152" s="5" t="s">
-        <v>1008</v>
-      </c>
-      <c r="J152" s="5" t="s">
-        <v>1009</v>
-      </c>
-      <c r="K152" s="5" t="s">
-        <v>1010</v>
       </c>
       <c r="L152" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M152" s="5" t="s">
-        <v>1011</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="153" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -9878,31 +9878,31 @@
         <v>7</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
       <c r="G153" s="6" t="s">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="H153" s="6" t="s">
         <v>278</v>
       </c>
       <c r="I153" s="6" t="s">
-        <v>1013</v>
+        <v>1007</v>
       </c>
       <c r="J153" s="6" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="K153" s="6" t="s">
-        <v>1015</v>
+        <v>1009</v>
       </c>
       <c r="L153" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M153" s="6" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="154" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -9913,34 +9913,34 @@
         <v>7</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
       <c r="F154" s="5"/>
       <c r="G154" s="5" t="s">
-        <v>1017</v>
+        <v>1011</v>
       </c>
       <c r="H154" s="5" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="I154" s="5" t="s">
-        <v>1019</v>
+        <v>1013</v>
       </c>
       <c r="J154" s="5" t="s">
-        <v>1020</v>
+        <v>1014</v>
       </c>
       <c r="K154" s="5" t="s">
-        <v>1021</v>
+        <v>1015</v>
       </c>
       <c r="L154" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M154" s="5" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="155" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="155" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -9948,33 +9948,33 @@
         <v>7</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
       <c r="D155" s="6"/>
-      <c r="E155" s="6"/>
-      <c r="F155" s="6" t="s">
-        <v>1024</v>
-      </c>
+      <c r="E155" s="9" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F155" s="6"/>
       <c r="G155" s="6" t="s">
-        <v>1025</v>
+        <v>1018</v>
       </c>
       <c r="H155" s="6" t="s">
-        <v>1026</v>
+        <v>1019</v>
       </c>
       <c r="I155" s="6" t="s">
-        <v>1027</v>
+        <v>1020</v>
       </c>
       <c r="J155" s="6" t="s">
-        <v>1028</v>
+        <v>1021</v>
       </c>
       <c r="K155" s="6" t="s">
-        <v>1029</v>
+        <v>1022</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M155" s="6" t="s">
-        <v>1030</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="156" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -9985,34 +9985,34 @@
         <v>7</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
       <c r="D156" s="5"/>
       <c r="E156" s="5"/>
       <c r="F156" s="5"/>
       <c r="G156" s="5" t="s">
-        <v>1031</v>
+        <v>1024</v>
       </c>
       <c r="H156" s="5" t="s">
-        <v>1032</v>
+        <v>1025</v>
       </c>
       <c r="I156" s="5" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="J156" s="5" t="s">
-        <v>1034</v>
+        <v>1027</v>
       </c>
       <c r="K156" s="5" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="L156" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M156" s="5" t="s">
-        <v>1036</v>
-      </c>
-    </row>
-    <row r="157" spans="1:13" ht="120" x14ac:dyDescent="0.25">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="157" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -10020,33 +10020,33 @@
         <v>7</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="D157" s="6"/>
-      <c r="E157" s="6"/>
-      <c r="F157" s="6" t="s">
-        <v>1038</v>
-      </c>
+      <c r="E157" s="9" t="s">
+        <v>1325</v>
+      </c>
+      <c r="F157" s="6"/>
       <c r="G157" s="6" t="s">
-        <v>1039</v>
+        <v>1031</v>
       </c>
       <c r="H157" s="6" t="s">
-        <v>1040</v>
+        <v>1032</v>
       </c>
       <c r="I157" s="6" t="s">
-        <v>1041</v>
+        <v>1033</v>
       </c>
       <c r="J157" s="6" t="s">
-        <v>1042</v>
+        <v>1034</v>
       </c>
       <c r="K157" s="6" t="s">
-        <v>1043</v>
+        <v>1035</v>
       </c>
       <c r="L157" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M157" s="6" t="s">
-        <v>1044</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="158" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10057,34 +10057,34 @@
         <v>7</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="D158" s="5"/>
       <c r="E158" s="5"/>
       <c r="F158" s="5"/>
       <c r="G158" s="5" t="s">
-        <v>1045</v>
+        <v>1037</v>
       </c>
       <c r="H158" s="5" t="s">
-        <v>1046</v>
+        <v>1038</v>
       </c>
       <c r="I158" s="5" t="s">
-        <v>1047</v>
+        <v>1039</v>
       </c>
       <c r="J158" s="5" t="s">
-        <v>1048</v>
+        <v>1040</v>
       </c>
       <c r="K158" s="5" t="s">
-        <v>1049</v>
+        <v>1041</v>
       </c>
       <c r="L158" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M158" s="5" t="s">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="159" spans="1:13" ht="195" x14ac:dyDescent="0.25">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="159" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -10092,33 +10092,33 @@
         <v>7</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>1051</v>
+        <v>1043</v>
       </c>
       <c r="D159" s="6"/>
-      <c r="E159" s="6"/>
-      <c r="F159" s="6" t="s">
-        <v>1052</v>
-      </c>
+      <c r="E159" s="9" t="s">
+        <v>1326</v>
+      </c>
+      <c r="F159" s="6"/>
       <c r="G159" s="6" t="s">
-        <v>1053</v>
+        <v>1044</v>
       </c>
       <c r="H159" s="6" t="s">
-        <v>1054</v>
+        <v>1045</v>
       </c>
       <c r="I159" s="6" t="s">
-        <v>1055</v>
+        <v>1046</v>
       </c>
       <c r="J159" s="6" t="s">
-        <v>1056</v>
+        <v>1047</v>
       </c>
       <c r="K159" s="6" t="s">
-        <v>1057</v>
+        <v>1048</v>
       </c>
       <c r="L159" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M159" s="6" t="s">
-        <v>1058</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="160" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10129,31 +10129,31 @@
         <v>7</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>1051</v>
+        <v>1043</v>
       </c>
       <c r="D160" s="5"/>
       <c r="E160" s="5"/>
       <c r="F160" s="5"/>
       <c r="G160" s="5" t="s">
-        <v>1059</v>
+        <v>1050</v>
       </c>
       <c r="H160" s="5" t="s">
-        <v>1060</v>
+        <v>1051</v>
       </c>
       <c r="I160" s="5" t="s">
-        <v>1061</v>
+        <v>1052</v>
       </c>
       <c r="J160" s="5" t="s">
-        <v>1062</v>
+        <v>1053</v>
       </c>
       <c r="K160" s="5" t="s">
-        <v>1063</v>
+        <v>1054</v>
       </c>
       <c r="L160" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M160" s="5" t="s">
-        <v>1064</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="161" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10164,31 +10164,31 @@
         <v>7</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>1051</v>
+        <v>1043</v>
       </c>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
       <c r="F161" s="6"/>
       <c r="G161" s="6" t="s">
-        <v>1065</v>
+        <v>1056</v>
       </c>
       <c r="H161" s="6" t="s">
-        <v>1066</v>
+        <v>1057</v>
       </c>
       <c r="I161" s="6" t="s">
-        <v>1067</v>
+        <v>1058</v>
       </c>
       <c r="J161" s="6" t="s">
-        <v>1068</v>
+        <v>1059</v>
       </c>
       <c r="K161" s="6" t="s">
-        <v>1069</v>
+        <v>1060</v>
       </c>
       <c r="L161" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M161" s="6" t="s">
-        <v>1070</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="162" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10199,34 +10199,34 @@
         <v>7</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>1051</v>
+        <v>1043</v>
       </c>
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
       <c r="F162" s="5"/>
       <c r="G162" s="5" t="s">
-        <v>1071</v>
+        <v>1062</v>
       </c>
       <c r="H162" s="5" t="s">
-        <v>1072</v>
+        <v>1063</v>
       </c>
       <c r="I162" s="5" t="s">
-        <v>1073</v>
+        <v>1064</v>
       </c>
       <c r="J162" s="5" t="s">
-        <v>1074</v>
+        <v>1065</v>
       </c>
       <c r="K162" s="5" t="s">
-        <v>1075</v>
+        <v>1066</v>
       </c>
       <c r="L162" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M162" s="5" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="163" spans="1:13" ht="255" x14ac:dyDescent="0.25">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="163" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -10234,33 +10234,33 @@
         <v>7</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>1077</v>
+        <v>1068</v>
       </c>
       <c r="D163" s="6"/>
-      <c r="E163" s="6"/>
-      <c r="F163" s="6" t="s">
-        <v>1078</v>
-      </c>
+      <c r="E163" s="9" t="s">
+        <v>1327</v>
+      </c>
+      <c r="F163" s="6"/>
       <c r="G163" s="6" t="s">
-        <v>1079</v>
+        <v>1069</v>
       </c>
       <c r="H163" s="6" t="s">
-        <v>1080</v>
+        <v>1070</v>
       </c>
       <c r="I163" s="6" t="s">
-        <v>1081</v>
+        <v>1071</v>
       </c>
       <c r="J163" s="6" t="s">
-        <v>1082</v>
+        <v>1072</v>
       </c>
       <c r="K163" s="6" t="s">
-        <v>1083</v>
+        <v>1073</v>
       </c>
       <c r="L163" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M163" s="6" t="s">
-        <v>1084</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="164" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10271,31 +10271,31 @@
         <v>7</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>1077</v>
+        <v>1068</v>
       </c>
       <c r="D164" s="5"/>
       <c r="E164" s="5"/>
       <c r="F164" s="5"/>
       <c r="G164" s="5" t="s">
-        <v>1085</v>
+        <v>1075</v>
       </c>
       <c r="H164" s="5" t="s">
-        <v>1086</v>
+        <v>1076</v>
       </c>
       <c r="I164" s="5" t="s">
-        <v>1087</v>
+        <v>1077</v>
       </c>
       <c r="J164" s="5" t="s">
-        <v>1088</v>
+        <v>1078</v>
       </c>
       <c r="K164" s="5" t="s">
-        <v>1089</v>
+        <v>1079</v>
       </c>
       <c r="L164" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M164" s="5" t="s">
-        <v>1090</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="165" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10306,31 +10306,31 @@
         <v>7</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>1077</v>
+        <v>1068</v>
       </c>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
       <c r="G165" s="6" t="s">
-        <v>1091</v>
+        <v>1081</v>
       </c>
       <c r="H165" s="6" t="s">
-        <v>1092</v>
+        <v>1082</v>
       </c>
       <c r="I165" s="6" t="s">
-        <v>1093</v>
+        <v>1083</v>
       </c>
       <c r="J165" s="6" t="s">
-        <v>1094</v>
+        <v>1084</v>
       </c>
       <c r="K165" s="6" t="s">
-        <v>1095</v>
+        <v>1085</v>
       </c>
       <c r="L165" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M165" s="6" t="s">
-        <v>1096</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="166" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -10341,34 +10341,34 @@
         <v>7</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>1077</v>
+        <v>1068</v>
       </c>
       <c r="D166" s="5"/>
       <c r="E166" s="5"/>
       <c r="F166" s="5"/>
       <c r="G166" s="5" t="s">
-        <v>1097</v>
+        <v>1087</v>
       </c>
       <c r="H166" s="5" t="s">
-        <v>1098</v>
+        <v>1088</v>
       </c>
       <c r="I166" s="5" t="s">
-        <v>1099</v>
+        <v>1089</v>
       </c>
       <c r="J166" s="5" t="s">
-        <v>1100</v>
+        <v>1090</v>
       </c>
       <c r="K166" s="5" t="s">
-        <v>1101</v>
+        <v>1091</v>
       </c>
       <c r="L166" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M166" s="5" t="s">
-        <v>1102</v>
-      </c>
-    </row>
-    <row r="167" spans="1:13" ht="165" x14ac:dyDescent="0.25">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="167" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -10376,33 +10376,33 @@
         <v>7</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>1103</v>
+        <v>1093</v>
       </c>
       <c r="D167" s="6"/>
-      <c r="E167" s="6"/>
-      <c r="F167" s="6" t="s">
-        <v>1104</v>
-      </c>
+      <c r="E167" s="9" t="s">
+        <v>1328</v>
+      </c>
+      <c r="F167" s="6"/>
       <c r="G167" s="6" t="s">
-        <v>1105</v>
+        <v>1094</v>
       </c>
       <c r="H167" s="6" t="s">
-        <v>1106</v>
+        <v>1095</v>
       </c>
       <c r="I167" s="6" t="s">
-        <v>1107</v>
+        <v>1096</v>
       </c>
       <c r="J167" s="6" t="s">
-        <v>1108</v>
+        <v>1097</v>
       </c>
       <c r="K167" s="6" t="s">
-        <v>1109</v>
+        <v>1098</v>
       </c>
       <c r="L167" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M167" s="6" t="s">
-        <v>1110</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="168" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10413,31 +10413,31 @@
         <v>7</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>1103</v>
+        <v>1093</v>
       </c>
       <c r="D168" s="5"/>
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
       <c r="G168" s="5" t="s">
-        <v>1111</v>
+        <v>1100</v>
       </c>
       <c r="H168" s="5" t="s">
-        <v>1112</v>
+        <v>1101</v>
       </c>
       <c r="I168" s="5" t="s">
-        <v>1113</v>
+        <v>1102</v>
       </c>
       <c r="J168" s="5" t="s">
-        <v>1114</v>
+        <v>1103</v>
       </c>
       <c r="K168" s="5" t="s">
-        <v>1115</v>
+        <v>1104</v>
       </c>
       <c r="L168" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M168" s="5" t="s">
-        <v>1116</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="169" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -10448,34 +10448,34 @@
         <v>7</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>1103</v>
+        <v>1093</v>
       </c>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6" t="s">
-        <v>1117</v>
+        <v>1106</v>
       </c>
       <c r="H169" s="6" t="s">
-        <v>1118</v>
+        <v>1107</v>
       </c>
       <c r="I169" s="6" t="s">
-        <v>1119</v>
+        <v>1108</v>
       </c>
       <c r="J169" s="6" t="s">
-        <v>1120</v>
+        <v>1109</v>
       </c>
       <c r="K169" s="6" t="s">
-        <v>1121</v>
+        <v>1110</v>
       </c>
       <c r="L169" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M169" s="6" t="s">
-        <v>1122</v>
-      </c>
-    </row>
-    <row r="170" spans="1:13" ht="195" x14ac:dyDescent="0.25">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="170" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A170" s="4">
         <v>169</v>
       </c>
@@ -10483,33 +10483,33 @@
         <v>7</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>1123</v>
+        <v>1112</v>
       </c>
       <c r="D170" s="5"/>
-      <c r="E170" s="5"/>
-      <c r="F170" s="5" t="s">
-        <v>1124</v>
-      </c>
+      <c r="E170" s="8" t="s">
+        <v>1329</v>
+      </c>
+      <c r="F170" s="5"/>
       <c r="G170" s="5" t="s">
-        <v>1125</v>
+        <v>1113</v>
       </c>
       <c r="H170" s="5" t="s">
-        <v>1126</v>
+        <v>1114</v>
       </c>
       <c r="I170" s="5" t="s">
-        <v>1127</v>
+        <v>1115</v>
       </c>
       <c r="J170" s="5" t="s">
-        <v>1128</v>
+        <v>1116</v>
       </c>
       <c r="K170" s="5" t="s">
-        <v>1129</v>
+        <v>1117</v>
       </c>
       <c r="L170" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M170" s="5" t="s">
-        <v>1130</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="171" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -10520,31 +10520,31 @@
         <v>7</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>1123</v>
+        <v>1112</v>
       </c>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
       <c r="G171" s="6" t="s">
-        <v>1131</v>
+        <v>1119</v>
       </c>
       <c r="H171" s="6" t="s">
-        <v>1132</v>
+        <v>1120</v>
       </c>
       <c r="I171" s="6" t="s">
-        <v>1133</v>
+        <v>1121</v>
       </c>
       <c r="J171" s="6" t="s">
-        <v>1134</v>
+        <v>1122</v>
       </c>
       <c r="K171" s="6" t="s">
-        <v>1135</v>
+        <v>1123</v>
       </c>
       <c r="L171" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M171" s="6" t="s">
-        <v>1136</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="172" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -10555,34 +10555,34 @@
         <v>7</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>1123</v>
+        <v>1112</v>
       </c>
       <c r="D172" s="5"/>
       <c r="E172" s="5"/>
       <c r="F172" s="5"/>
       <c r="G172" s="5" t="s">
-        <v>1137</v>
+        <v>1125</v>
       </c>
       <c r="H172" s="5" t="s">
-        <v>1138</v>
+        <v>1126</v>
       </c>
       <c r="I172" s="5" t="s">
-        <v>1139</v>
+        <v>1127</v>
       </c>
       <c r="J172" s="5" t="s">
-        <v>1140</v>
+        <v>1128</v>
       </c>
       <c r="K172" s="5" t="s">
-        <v>1141</v>
+        <v>1129</v>
       </c>
       <c r="L172" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M172" s="5" t="s">
-        <v>1142</v>
-      </c>
-    </row>
-    <row r="173" spans="1:13" ht="240" x14ac:dyDescent="0.25">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="173" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>172</v>
       </c>
@@ -10590,33 +10590,33 @@
         <v>7</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>1143</v>
+        <v>1131</v>
       </c>
       <c r="D173" s="6"/>
-      <c r="E173" s="6"/>
-      <c r="F173" s="6" t="s">
-        <v>1144</v>
-      </c>
+      <c r="E173" s="9" t="s">
+        <v>1330</v>
+      </c>
+      <c r="F173" s="6"/>
       <c r="G173" s="6" t="s">
-        <v>1145</v>
+        <v>1132</v>
       </c>
       <c r="H173" s="6" t="s">
-        <v>1146</v>
+        <v>1133</v>
       </c>
       <c r="I173" s="6" t="s">
-        <v>1147</v>
+        <v>1134</v>
       </c>
       <c r="J173" s="6" t="s">
-        <v>1148</v>
+        <v>1135</v>
       </c>
       <c r="K173" s="6" t="s">
-        <v>1149</v>
+        <v>1136</v>
       </c>
       <c r="L173" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M173" s="6" t="s">
-        <v>1150</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="174" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10627,31 +10627,31 @@
         <v>7</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>1143</v>
+        <v>1131</v>
       </c>
       <c r="D174" s="5"/>
       <c r="E174" s="5"/>
       <c r="F174" s="5"/>
       <c r="G174" s="5" t="s">
-        <v>1151</v>
+        <v>1138</v>
       </c>
       <c r="H174" s="5" t="s">
-        <v>1152</v>
+        <v>1139</v>
       </c>
       <c r="I174" s="5" t="s">
-        <v>1153</v>
+        <v>1140</v>
       </c>
       <c r="J174" s="5" t="s">
-        <v>1154</v>
+        <v>1141</v>
       </c>
       <c r="K174" s="5" t="s">
-        <v>1155</v>
+        <v>1142</v>
       </c>
       <c r="L174" s="4" t="s">
         <v>32</v>
       </c>
       <c r="M174" s="5" t="s">
-        <v>1156</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="175" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10662,31 +10662,31 @@
         <v>7</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>1143</v>
+        <v>1131</v>
       </c>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
       <c r="F175" s="6"/>
       <c r="G175" s="6" t="s">
-        <v>1157</v>
+        <v>1144</v>
       </c>
       <c r="H175" s="6" t="s">
-        <v>1158</v>
+        <v>1145</v>
       </c>
       <c r="I175" s="6" t="s">
-        <v>1159</v>
+        <v>1146</v>
       </c>
       <c r="J175" s="6" t="s">
-        <v>1160</v>
+        <v>1147</v>
       </c>
       <c r="K175" s="6" t="s">
-        <v>1161</v>
+        <v>1148</v>
       </c>
       <c r="L175" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M175" s="6" t="s">
-        <v>1162</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="176" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -10697,34 +10697,34 @@
         <v>7</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>1143</v>
+        <v>1131</v>
       </c>
       <c r="D176" s="5"/>
       <c r="E176" s="5"/>
       <c r="F176" s="5"/>
       <c r="G176" s="5" t="s">
-        <v>1163</v>
+        <v>1150</v>
       </c>
       <c r="H176" s="5" t="s">
-        <v>1138</v>
+        <v>1126</v>
       </c>
       <c r="I176" s="5" t="s">
-        <v>1139</v>
+        <v>1127</v>
       </c>
       <c r="J176" s="5" t="s">
-        <v>1140</v>
+        <v>1128</v>
       </c>
       <c r="K176" s="5" t="s">
-        <v>1141</v>
+        <v>1129</v>
       </c>
       <c r="L176" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M176" s="5" t="s">
-        <v>1164</v>
-      </c>
-    </row>
-    <row r="177" spans="1:13" ht="240" x14ac:dyDescent="0.25">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="177" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>176</v>
       </c>
@@ -10732,33 +10732,33 @@
         <v>7</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>1165</v>
+        <v>1152</v>
       </c>
       <c r="D177" s="6"/>
-      <c r="E177" s="6"/>
-      <c r="F177" s="6" t="s">
-        <v>1166</v>
-      </c>
+      <c r="E177" s="6" t="s">
+        <v>1331</v>
+      </c>
+      <c r="F177" s="6"/>
       <c r="G177" s="6" t="s">
-        <v>1167</v>
+        <v>1153</v>
       </c>
       <c r="H177" s="6" t="s">
-        <v>1168</v>
+        <v>1154</v>
       </c>
       <c r="I177" s="6" t="s">
-        <v>1169</v>
+        <v>1155</v>
       </c>
       <c r="J177" s="6" t="s">
-        <v>1170</v>
+        <v>1156</v>
       </c>
       <c r="K177" s="6" t="s">
-        <v>1171</v>
+        <v>1157</v>
       </c>
       <c r="L177" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M177" s="6" t="s">
-        <v>1172</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="178" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10769,31 +10769,31 @@
         <v>7</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>1165</v>
+        <v>1152</v>
       </c>
       <c r="D178" s="5"/>
       <c r="E178" s="5"/>
       <c r="F178" s="5"/>
       <c r="G178" s="5" t="s">
-        <v>1173</v>
+        <v>1159</v>
       </c>
       <c r="H178" s="5" t="s">
-        <v>1174</v>
+        <v>1160</v>
       </c>
       <c r="I178" s="5" t="s">
-        <v>1175</v>
+        <v>1161</v>
       </c>
       <c r="J178" s="5" t="s">
-        <v>1176</v>
+        <v>1162</v>
       </c>
       <c r="K178" s="5" t="s">
-        <v>1177</v>
+        <v>1163</v>
       </c>
       <c r="L178" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M178" s="5" t="s">
-        <v>1178</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="179" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -10804,31 +10804,31 @@
         <v>7</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>1165</v>
+        <v>1152</v>
       </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
       <c r="G179" s="6" t="s">
-        <v>1179</v>
+        <v>1165</v>
       </c>
       <c r="H179" s="6" t="s">
-        <v>1180</v>
+        <v>1166</v>
       </c>
       <c r="I179" s="6" t="s">
-        <v>1181</v>
+        <v>1167</v>
       </c>
       <c r="J179" s="6" t="s">
-        <v>1182</v>
+        <v>1168</v>
       </c>
       <c r="K179" s="6" t="s">
-        <v>1183</v>
+        <v>1169</v>
       </c>
       <c r="L179" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M179" s="6" t="s">
-        <v>1184</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="180" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -10839,31 +10839,31 @@
         <v>7</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>1165</v>
+        <v>1152</v>
       </c>
       <c r="D180" s="5"/>
       <c r="E180" s="5"/>
       <c r="F180" s="5"/>
       <c r="G180" s="5" t="s">
-        <v>1185</v>
+        <v>1171</v>
       </c>
       <c r="H180" s="5" t="s">
-        <v>1186</v>
+        <v>1172</v>
       </c>
       <c r="I180" s="5" t="s">
-        <v>1187</v>
+        <v>1173</v>
       </c>
       <c r="J180" s="5" t="s">
-        <v>1188</v>
+        <v>1174</v>
       </c>
       <c r="K180" s="5" t="s">
-        <v>1189</v>
+        <v>1175</v>
       </c>
       <c r="L180" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M180" s="5" t="s">
-        <v>1190</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="181" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -10874,34 +10874,34 @@
         <v>7</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>1165</v>
+        <v>1152</v>
       </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
       <c r="F181" s="6"/>
       <c r="G181" s="6" t="s">
-        <v>1191</v>
+        <v>1177</v>
       </c>
       <c r="H181" s="6" t="s">
-        <v>1192</v>
+        <v>1178</v>
       </c>
       <c r="I181" s="6" t="s">
-        <v>1193</v>
+        <v>1179</v>
       </c>
       <c r="J181" s="6" t="s">
-        <v>1194</v>
+        <v>1180</v>
       </c>
       <c r="K181" s="6" t="s">
-        <v>1195</v>
+        <v>1181</v>
       </c>
       <c r="L181" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M181" s="6" t="s">
-        <v>1196</v>
-      </c>
-    </row>
-    <row r="182" spans="1:13" ht="210" x14ac:dyDescent="0.25">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="182" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A182" s="4">
         <v>181</v>
       </c>
@@ -10909,33 +10909,33 @@
         <v>7</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>1197</v>
+        <v>1183</v>
       </c>
       <c r="D182" s="5"/>
-      <c r="E182" s="5"/>
-      <c r="F182" s="5" t="s">
-        <v>1198</v>
-      </c>
+      <c r="E182" s="5" t="s">
+        <v>1332</v>
+      </c>
+      <c r="F182" s="5"/>
       <c r="G182" s="5" t="s">
-        <v>1199</v>
+        <v>1184</v>
       </c>
       <c r="H182" s="5" t="s">
-        <v>1200</v>
+        <v>1185</v>
       </c>
       <c r="I182" s="5" t="s">
-        <v>1201</v>
+        <v>1186</v>
       </c>
       <c r="J182" s="5" t="s">
-        <v>1202</v>
+        <v>1187</v>
       </c>
       <c r="K182" s="5" t="s">
-        <v>1203</v>
+        <v>1188</v>
       </c>
       <c r="L182" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M182" s="5" t="s">
-        <v>1204</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="183" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -10946,31 +10946,31 @@
         <v>7</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>1197</v>
+        <v>1183</v>
       </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6" t="s">
-        <v>1205</v>
+        <v>1190</v>
       </c>
       <c r="H183" s="6" t="s">
-        <v>1206</v>
+        <v>1191</v>
       </c>
       <c r="I183" s="6" t="s">
-        <v>1207</v>
+        <v>1192</v>
       </c>
       <c r="J183" s="6" t="s">
-        <v>1208</v>
+        <v>1193</v>
       </c>
       <c r="K183" s="6" t="s">
-        <v>1209</v>
+        <v>1194</v>
       </c>
       <c r="L183" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M183" s="6" t="s">
-        <v>1210</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="184" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -10981,31 +10981,31 @@
         <v>7</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>1197</v>
+        <v>1183</v>
       </c>
       <c r="D184" s="5"/>
       <c r="E184" s="5"/>
       <c r="F184" s="5"/>
       <c r="G184" s="5" t="s">
-        <v>1211</v>
+        <v>1196</v>
       </c>
       <c r="H184" s="5" t="s">
-        <v>1212</v>
+        <v>1197</v>
       </c>
       <c r="I184" s="5" t="s">
-        <v>1213</v>
+        <v>1198</v>
       </c>
       <c r="J184" s="5" t="s">
-        <v>1214</v>
+        <v>1199</v>
       </c>
       <c r="K184" s="5" t="s">
-        <v>1215</v>
+        <v>1200</v>
       </c>
       <c r="L184" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M184" s="5" t="s">
-        <v>1216</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="185" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -11016,31 +11016,31 @@
         <v>7</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>1197</v>
+        <v>1183</v>
       </c>
       <c r="D185" s="6"/>
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
       <c r="G185" s="6" t="s">
-        <v>1217</v>
+        <v>1202</v>
       </c>
       <c r="H185" s="6" t="s">
-        <v>1218</v>
+        <v>1203</v>
       </c>
       <c r="I185" s="6" t="s">
-        <v>1219</v>
+        <v>1204</v>
       </c>
       <c r="J185" s="6" t="s">
-        <v>1220</v>
+        <v>1205</v>
       </c>
       <c r="K185" s="6" t="s">
-        <v>1221</v>
+        <v>1206</v>
       </c>
       <c r="L185" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M185" s="6" t="s">
-        <v>1222</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="186" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -11051,34 +11051,34 @@
         <v>7</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>1197</v>
+        <v>1183</v>
       </c>
       <c r="D186" s="5"/>
       <c r="E186" s="5"/>
       <c r="F186" s="5"/>
       <c r="G186" s="5" t="s">
-        <v>1223</v>
+        <v>1208</v>
       </c>
       <c r="H186" s="5" t="s">
-        <v>1224</v>
+        <v>1209</v>
       </c>
       <c r="I186" s="5" t="s">
-        <v>1225</v>
+        <v>1210</v>
       </c>
       <c r="J186" s="5" t="s">
-        <v>1226</v>
+        <v>1211</v>
       </c>
       <c r="K186" s="5" t="s">
-        <v>1227</v>
+        <v>1212</v>
       </c>
       <c r="L186" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M186" s="5" t="s">
-        <v>1228</v>
-      </c>
-    </row>
-    <row r="187" spans="1:13" ht="180" x14ac:dyDescent="0.25">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="187" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
         <v>186</v>
       </c>
@@ -11086,33 +11086,33 @@
         <v>7</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>1229</v>
+        <v>1214</v>
       </c>
       <c r="D187" s="6"/>
-      <c r="E187" s="6"/>
-      <c r="F187" s="6" t="s">
-        <v>1230</v>
-      </c>
+      <c r="E187" s="6" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F187" s="6"/>
       <c r="G187" s="6" t="s">
-        <v>1231</v>
+        <v>1215</v>
       </c>
       <c r="H187" s="6" t="s">
-        <v>1232</v>
+        <v>1216</v>
       </c>
       <c r="I187" s="6" t="s">
-        <v>1233</v>
+        <v>1217</v>
       </c>
       <c r="J187" s="6" t="s">
-        <v>1234</v>
+        <v>1218</v>
       </c>
       <c r="K187" s="6" t="s">
-        <v>1235</v>
+        <v>1219</v>
       </c>
       <c r="L187" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M187" s="6" t="s">
-        <v>1236</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="188" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11123,31 +11123,31 @@
         <v>7</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>1229</v>
+        <v>1214</v>
       </c>
       <c r="D188" s="5"/>
       <c r="E188" s="5"/>
       <c r="F188" s="5"/>
       <c r="G188" s="5" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="H188" s="5" t="s">
-        <v>1237</v>
+        <v>1221</v>
       </c>
       <c r="I188" s="5" t="s">
-        <v>1238</v>
+        <v>1222</v>
       </c>
       <c r="J188" s="5" t="s">
-        <v>1239</v>
+        <v>1223</v>
       </c>
       <c r="K188" s="5" t="s">
-        <v>1240</v>
+        <v>1224</v>
       </c>
       <c r="L188" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M188" s="5" t="s">
-        <v>1241</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="189" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -11158,31 +11158,31 @@
         <v>7</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>1229</v>
+        <v>1214</v>
       </c>
       <c r="D189" s="6"/>
       <c r="E189" s="6"/>
       <c r="F189" s="6"/>
       <c r="G189" s="6" t="s">
-        <v>1242</v>
+        <v>1226</v>
       </c>
       <c r="H189" s="6" t="s">
-        <v>1243</v>
+        <v>1227</v>
       </c>
       <c r="I189" s="6" t="s">
-        <v>1244</v>
+        <v>1228</v>
       </c>
       <c r="J189" s="6" t="s">
-        <v>1245</v>
+        <v>1229</v>
       </c>
       <c r="K189" s="6" t="s">
-        <v>1246</v>
+        <v>1230</v>
       </c>
       <c r="L189" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M189" s="6" t="s">
-        <v>1247</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="190" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11193,31 +11193,31 @@
         <v>7</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>1229</v>
+        <v>1214</v>
       </c>
       <c r="D190" s="5"/>
       <c r="E190" s="5"/>
       <c r="F190" s="5"/>
       <c r="G190" s="5" t="s">
-        <v>1248</v>
+        <v>1232</v>
       </c>
       <c r="H190" s="5" t="s">
-        <v>1249</v>
+        <v>1233</v>
       </c>
       <c r="I190" s="5" t="s">
-        <v>1250</v>
+        <v>1234</v>
       </c>
       <c r="J190" s="5" t="s">
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="K190" s="5" t="s">
-        <v>1252</v>
+        <v>1236</v>
       </c>
       <c r="L190" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M190" s="5" t="s">
-        <v>1253</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="191" spans="1:13" ht="90" x14ac:dyDescent="0.25">
@@ -11228,34 +11228,34 @@
         <v>7</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>1229</v>
+        <v>1214</v>
       </c>
       <c r="D191" s="6"/>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
       <c r="G191" s="6" t="s">
-        <v>1254</v>
+        <v>1238</v>
       </c>
       <c r="H191" s="6" t="s">
-        <v>1255</v>
+        <v>1239</v>
       </c>
       <c r="I191" s="6" t="s">
-        <v>1256</v>
+        <v>1240</v>
       </c>
       <c r="J191" s="6" t="s">
-        <v>1257</v>
+        <v>1241</v>
       </c>
       <c r="K191" s="6" t="s">
-        <v>1258</v>
+        <v>1242</v>
       </c>
       <c r="L191" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M191" s="6" t="s">
-        <v>1259</v>
-      </c>
-    </row>
-    <row r="192" spans="1:13" ht="240" x14ac:dyDescent="0.25">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="192" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A192" s="4">
         <v>191</v>
       </c>
@@ -11263,33 +11263,33 @@
         <v>7</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="D192" s="5"/>
-      <c r="E192" s="5"/>
-      <c r="F192" s="5" t="s">
-        <v>1261</v>
-      </c>
+      <c r="E192" s="5" t="s">
+        <v>1334</v>
+      </c>
+      <c r="F192" s="5"/>
       <c r="G192" s="5" t="s">
-        <v>1262</v>
+        <v>1245</v>
       </c>
       <c r="H192" s="5" t="s">
-        <v>1263</v>
+        <v>1246</v>
       </c>
       <c r="I192" s="5" t="s">
-        <v>1264</v>
+        <v>1247</v>
       </c>
       <c r="J192" s="5" t="s">
-        <v>1265</v>
+        <v>1248</v>
       </c>
       <c r="K192" s="5" t="s">
-        <v>1266</v>
+        <v>1249</v>
       </c>
       <c r="L192" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M192" s="5" t="s">
-        <v>1267</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="193" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11300,31 +11300,31 @@
         <v>7</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="D193" s="6"/>
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
       <c r="G193" s="6" t="s">
-        <v>1268</v>
+        <v>1251</v>
       </c>
       <c r="H193" s="6" t="s">
-        <v>1269</v>
+        <v>1252</v>
       </c>
       <c r="I193" s="6" t="s">
-        <v>1270</v>
+        <v>1253</v>
       </c>
       <c r="J193" s="6" t="s">
-        <v>1271</v>
+        <v>1254</v>
       </c>
       <c r="K193" s="6" t="s">
-        <v>1272</v>
+        <v>1255</v>
       </c>
       <c r="L193" s="2" t="s">
         <v>39</v>
       </c>
       <c r="M193" s="6" t="s">
-        <v>1273</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="194" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11335,31 +11335,31 @@
         <v>7</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="D194" s="5"/>
       <c r="E194" s="5"/>
       <c r="F194" s="5"/>
       <c r="G194" s="5" t="s">
-        <v>1274</v>
+        <v>1257</v>
       </c>
       <c r="H194" s="5" t="s">
-        <v>1275</v>
+        <v>1258</v>
       </c>
       <c r="I194" s="5" t="s">
-        <v>1276</v>
+        <v>1259</v>
       </c>
       <c r="J194" s="5" t="s">
-        <v>1277</v>
+        <v>1260</v>
       </c>
       <c r="K194" s="5" t="s">
-        <v>1278</v>
+        <v>1261</v>
       </c>
       <c r="L194" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M194" s="5" t="s">
-        <v>1279</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="195" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -11370,31 +11370,31 @@
         <v>7</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="D195" s="6"/>
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
       <c r="G195" s="6" t="s">
-        <v>1280</v>
+        <v>1263</v>
       </c>
       <c r="H195" s="6" t="s">
-        <v>1281</v>
+        <v>1264</v>
       </c>
       <c r="I195" s="6" t="s">
-        <v>1282</v>
+        <v>1265</v>
       </c>
       <c r="J195" s="6" t="s">
-        <v>1283</v>
+        <v>1266</v>
       </c>
       <c r="K195" s="6" t="s">
-        <v>1284</v>
+        <v>1267</v>
       </c>
       <c r="L195" s="2" t="s">
         <v>52</v>
       </c>
       <c r="M195" s="6" t="s">
-        <v>1285</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="196" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11405,34 +11405,34 @@
         <v>7</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
       <c r="D196" s="5"/>
       <c r="E196" s="5"/>
       <c r="F196" s="5"/>
       <c r="G196" s="5" t="s">
-        <v>1286</v>
+        <v>1269</v>
       </c>
       <c r="H196" s="5" t="s">
-        <v>1287</v>
+        <v>1270</v>
       </c>
       <c r="I196" s="5" t="s">
-        <v>1288</v>
+        <v>1271</v>
       </c>
       <c r="J196" s="5" t="s">
-        <v>1289</v>
+        <v>1272</v>
       </c>
       <c r="K196" s="5" t="s">
-        <v>1290</v>
+        <v>1273</v>
       </c>
       <c r="L196" s="4" t="s">
         <v>25</v>
       </c>
       <c r="M196" s="5" t="s">
-        <v>1291</v>
-      </c>
-    </row>
-    <row r="197" spans="1:13" ht="270" x14ac:dyDescent="0.25">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="197" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>196</v>
       </c>
@@ -11440,33 +11440,33 @@
         <v>7</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>1292</v>
+        <v>1275</v>
       </c>
       <c r="D197" s="6"/>
-      <c r="E197" s="6"/>
-      <c r="F197" s="6" t="s">
-        <v>1293</v>
-      </c>
+      <c r="E197" s="6" t="s">
+        <v>1335</v>
+      </c>
+      <c r="F197" s="6"/>
       <c r="G197" s="6" t="s">
-        <v>1294</v>
+        <v>1276</v>
       </c>
       <c r="H197" s="6" t="s">
-        <v>1295</v>
+        <v>1277</v>
       </c>
       <c r="I197" s="6" t="s">
-        <v>1296</v>
+        <v>1278</v>
       </c>
       <c r="J197" s="6" t="s">
-        <v>1297</v>
+        <v>1279</v>
       </c>
       <c r="K197" s="6" t="s">
-        <v>1298</v>
+        <v>1280</v>
       </c>
       <c r="L197" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M197" s="6" t="s">
-        <v>1299</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="198" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -11477,31 +11477,31 @@
         <v>7</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>1292</v>
+        <v>1275</v>
       </c>
       <c r="D198" s="5"/>
       <c r="E198" s="5"/>
       <c r="F198" s="5"/>
       <c r="G198" s="5" t="s">
-        <v>1300</v>
+        <v>1282</v>
       </c>
       <c r="H198" s="5" t="s">
-        <v>1301</v>
+        <v>1283</v>
       </c>
       <c r="I198" s="5" t="s">
-        <v>1302</v>
+        <v>1284</v>
       </c>
       <c r="J198" s="5" t="s">
-        <v>1303</v>
+        <v>1285</v>
       </c>
       <c r="K198" s="5" t="s">
-        <v>1304</v>
+        <v>1286</v>
       </c>
       <c r="L198" s="4" t="s">
         <v>52</v>
       </c>
       <c r="M198" s="5" t="s">
-        <v>1305</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="199" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -11512,31 +11512,31 @@
         <v>7</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>1292</v>
+        <v>1275</v>
       </c>
       <c r="D199" s="6"/>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
       <c r="G199" s="6" t="s">
-        <v>1306</v>
+        <v>1288</v>
       </c>
       <c r="H199" s="6" t="s">
-        <v>1307</v>
+        <v>1289</v>
       </c>
       <c r="I199" s="6" t="s">
-        <v>1308</v>
+        <v>1290</v>
       </c>
       <c r="J199" s="6" t="s">
-        <v>1309</v>
+        <v>1291</v>
       </c>
       <c r="K199" s="6" t="s">
-        <v>1310</v>
+        <v>1292</v>
       </c>
       <c r="L199" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M199" s="6" t="s">
-        <v>1311</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="200" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -11547,31 +11547,31 @@
         <v>7</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>1292</v>
+        <v>1275</v>
       </c>
       <c r="D200" s="5"/>
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
       <c r="G200" s="5" t="s">
-        <v>1312</v>
+        <v>1294</v>
       </c>
       <c r="H200" s="5" t="s">
-        <v>1313</v>
+        <v>1295</v>
       </c>
       <c r="I200" s="5" t="s">
-        <v>1314</v>
+        <v>1296</v>
       </c>
       <c r="J200" s="5" t="s">
-        <v>1315</v>
+        <v>1297</v>
       </c>
       <c r="K200" s="5" t="s">
-        <v>1316</v>
+        <v>1298</v>
       </c>
       <c r="L200" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M200" s="5" t="s">
-        <v>1317</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="201" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -11582,31 +11582,31 @@
         <v>7</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>1292</v>
+        <v>1275</v>
       </c>
       <c r="D201" s="6"/>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
       <c r="G201" s="6" t="s">
-        <v>1318</v>
+        <v>1300</v>
       </c>
       <c r="H201" s="6" t="s">
-        <v>1319</v>
+        <v>1301</v>
       </c>
       <c r="I201" s="6" t="s">
-        <v>1320</v>
+        <v>1302</v>
       </c>
       <c r="J201" s="6" t="s">
-        <v>1321</v>
+        <v>1303</v>
       </c>
       <c r="K201" s="6" t="s">
-        <v>1322</v>
+        <v>1304</v>
       </c>
       <c r="L201" s="2" t="s">
         <v>32</v>
       </c>
       <c r="M201" s="6" t="s">
-        <v>1323</v>
+        <v>1305</v>
       </c>
     </row>
   </sheetData>
@@ -11622,6 +11622,19 @@
     <hyperlink ref="E97" r:id="rId9"/>
     <hyperlink ref="E100" r:id="rId10"/>
     <hyperlink ref="E132" r:id="rId11"/>
+    <hyperlink ref="E136" r:id="rId12"/>
+    <hyperlink ref="E140" r:id="rId13"/>
+    <hyperlink ref="E144" r:id="rId14"/>
+    <hyperlink ref="E148" r:id="rId15"/>
+    <hyperlink ref="E150" r:id="rId16"/>
+    <hyperlink ref="E152" r:id="rId17"/>
+    <hyperlink ref="E155" r:id="rId18"/>
+    <hyperlink ref="E157" r:id="rId19"/>
+    <hyperlink ref="E159" r:id="rId20"/>
+    <hyperlink ref="E163" r:id="rId21"/>
+    <hyperlink ref="E167" r:id="rId22"/>
+    <hyperlink ref="E170" r:id="rId23"/>
+    <hyperlink ref="E173" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Thiet ke trang luyen de v17
</commit_message>
<xml_diff>
--- a/ETS2023_Test1_Final_Architecture.xlsx
+++ b/ETS2023_Test1_Final_Architecture.xlsx
@@ -4030,7 +4030,7 @@
     <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(3).png</t>
   </si>
   <si>
-    <t>https://github.com/bangvang1105-tech/Audio-Test-1-ETS-2023/raw/refs/heads/main/Test%201%20ETS%202023.mp3</t>
+    <t>https://drive.google.com/file/d/14yGl8HQLGWVQRJ9wKb3tllrgH0prTzdC/view?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -4502,9 +4502,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Thiet ke trang luyen de v21
</commit_message>
<xml_diff>
--- a/ETS2023_Test1_Final_Architecture.xlsx
+++ b/ETS2023_Test1_Final_Architecture.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28035" windowHeight="11730"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28035" windowHeight="11730" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Info" sheetId="1" r:id="rId1"/>
@@ -3940,97 +3940,97 @@
     <t>Giải thích: Maria viết trong email thứ 2 rằng: Ông Eklund thích tất cả bài viết của bà, và tất nhiên là CẢ bài báo/review gần đây về cuốn tự truyện của ông ấy ('your recent article about The Theatre Lights Dimmed!') -&gt; Ông ấy hài lòng với bài review của Joshi.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/main/p1_01.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p1_02.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p1_03.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p1_04.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p1_05.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p1_06.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p3_63.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p3_66.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p3_69.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p4_96.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p4_99.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_131.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_135.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_139.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p6_143.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_147.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_149.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_151.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_154.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_156.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_158.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_162.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_166.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_169.png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_172.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_176(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_176(2).png </t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_181(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_181(2).png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_186(3).png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_191(3).png</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-1-ETS-2023/refs/heads/main/p7_196(3).png</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/14yGl8HQLGWVQRJ9wKb3tllrgH0prTzdC/view?usp=sharing</t>
+    <t>https://res.cloudinary.com/dhmq07vzk/video/upload/v1782455168/Test_1_ETS_2023_vfth4v.mp3</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458761/p1_01_TEST_1_2023_ucgyk7.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458762/p1_02_1_TEST_1_2023_dolohs.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458762/p1_03_TEST_1_2023_zrrqff.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458763/p1_04_TEST_1_2023_yo8ngp.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458762/p1_05_TEST_1_2023_qwnvqc.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458764/p1_06_TEST_1_2023_pcjhdq.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458763/p3_63_TEST_1_2023_ceizvb.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458764/p3_66_TEST_1_2023_am2aqa.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458764/p3_69_TEST_1_2023_dizo4n.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458765/p4_96_TEST_1_2023_qf2sov.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458766/p4_99_TEST_1_2023_okannw.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458766/p6_131_TEST_1_2023_cexxzd.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458767/p6_135_TEST_1_2023_mrrxxf.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458767/p6_139_TEST_1_2023_j6kmzj.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458768/p6_143_TEST_1_2023_z8o89q.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458769/p7_147_TEST_1_2023_lmkhip.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458769/p7_149_TEST_1_2023_s8vtob.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458770/p7_151_TEST_1_2023_nftbes.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458771/p7_154_TEST_1_2023_cjxafh.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458771/p7_156_TEST_1_2023_b3grmc.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458772/p7_158_TEST_1_2023_zpi9f2.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458772/p7_162_TEST_1_2023_dawwpa.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458773/p7_166_TEST_1_2023_q3ybno.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458774/p7_169_TEST_1_2023_txcpwm.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458774/p7_172_TEST_1_2023_y4z6nx.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458775/p7_176_1_TEST_1_2023_pnyl3i.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458775/p7_176_2_TEST_1_2023_qi068t.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458776/p7_181_1_TEST_1_2023_rsoqhe.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458777/p7_181_2_TEST_1_2023_gth3hp.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458777/p7_186_1_TEST_1_2023_eibrkr.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458778/p7_186_2_TEST_1_2023_whucss.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458778/p7_186_3_TEST_1_2023_vystwu.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458779/p7_191_1_TEST_1_2023_sxe8v9.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458780/p7_191_2_TEST_1_2023_onmrvc.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458780/p7_191_3_TEST_1_2023_kc7ifg.png</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458781/p7_196_1_TEST_1_2023_cmfmak.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458782/p7_196_2_TEST_1_2023_kjianl.png | https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458782/p7_196_3_TEST_1_2023_vrlvt5.png</t>
   </si>
 </sst>
 </file>
@@ -4146,15 +4146,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4491,8 +4489,8 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>1336</v>
+      <c r="C2" s="9" t="s">
+        <v>1306</v>
       </c>
       <c r="D2" s="2">
         <v>120</v>
@@ -4502,6 +4500,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4573,8 +4574,8 @@
         <v>20</v>
       </c>
       <c r="D2" s="5"/>
-      <c r="E2" s="8" t="s">
-        <v>1306</v>
+      <c r="E2" s="7" t="s">
+        <v>1307</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
@@ -4597,7 +4598,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -4608,8 +4609,8 @@
         <v>27</v>
       </c>
       <c r="D3" s="6"/>
-      <c r="E3" s="9" t="s">
-        <v>1307</v>
+      <c r="E3" s="8" t="s">
+        <v>1308</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -4632,7 +4633,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -4643,8 +4644,8 @@
         <v>34</v>
       </c>
       <c r="D4" s="5"/>
-      <c r="E4" s="8" t="s">
-        <v>1308</v>
+      <c r="E4" s="7" t="s">
+        <v>1309</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
@@ -4667,7 +4668,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -4678,8 +4679,8 @@
         <v>41</v>
       </c>
       <c r="D5" s="6"/>
-      <c r="E5" s="9" t="s">
-        <v>1309</v>
+      <c r="E5" s="8" t="s">
+        <v>1310</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -4702,7 +4703,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -4713,8 +4714,8 @@
         <v>47</v>
       </c>
       <c r="D6" s="5"/>
-      <c r="E6" s="8" t="s">
-        <v>1310</v>
+      <c r="E6" s="7" t="s">
+        <v>1311</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
@@ -4737,7 +4738,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -4748,8 +4749,8 @@
         <v>54</v>
       </c>
       <c r="D7" s="6"/>
-      <c r="E7" s="9" t="s">
-        <v>1311</v>
+      <c r="E7" s="8" t="s">
+        <v>1312</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
@@ -6678,7 +6679,7 @@
         <v>408</v>
       </c>
       <c r="D63" s="6"/>
-      <c r="E63" s="9"/>
+      <c r="E63" s="8"/>
       <c r="F63" s="6" t="s">
         <v>409</v>
       </c>
@@ -6704,7 +6705,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -6715,8 +6716,8 @@
         <v>408</v>
       </c>
       <c r="D64" s="5"/>
-      <c r="E64" s="8" t="s">
-        <v>1312</v>
+      <c r="E64" s="7" t="s">
+        <v>1313</v>
       </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5" t="s">
@@ -6813,7 +6814,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -6824,8 +6825,8 @@
         <v>427</v>
       </c>
       <c r="D67" s="6"/>
-      <c r="E67" s="9" t="s">
-        <v>1313</v>
+      <c r="E67" s="8" t="s">
+        <v>1314</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
@@ -6922,7 +6923,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -6933,8 +6934,8 @@
         <v>447</v>
       </c>
       <c r="D70" s="5"/>
-      <c r="E70" s="8" t="s">
-        <v>1314</v>
+      <c r="E70" s="7" t="s">
+        <v>1315</v>
       </c>
       <c r="F70" s="5"/>
       <c r="G70" s="5" t="s">
@@ -7887,7 +7888,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="97" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -7898,8 +7899,8 @@
         <v>627</v>
       </c>
       <c r="D97" s="6"/>
-      <c r="E97" s="9" t="s">
-        <v>1315</v>
+      <c r="E97" s="8" t="s">
+        <v>1316</v>
       </c>
       <c r="F97" s="6"/>
       <c r="G97" s="6" t="s">
@@ -7996,7 +7997,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -8007,8 +8008,8 @@
         <v>647</v>
       </c>
       <c r="D100" s="5"/>
-      <c r="E100" s="8" t="s">
-        <v>1316</v>
+      <c r="E100" s="7" t="s">
+        <v>1317</v>
       </c>
       <c r="F100" s="5"/>
       <c r="G100" s="5" t="s">
@@ -9129,8 +9130,8 @@
         <v>876</v>
       </c>
       <c r="D132" s="5"/>
-      <c r="E132" s="8" t="s">
-        <v>1317</v>
+      <c r="E132" s="7" t="s">
+        <v>1318</v>
       </c>
       <c r="F132" s="5"/>
       <c r="G132" s="5" t="s">
@@ -9260,7 +9261,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="136" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>135</v>
       </c>
@@ -9271,8 +9272,8 @@
         <v>901</v>
       </c>
       <c r="D136" s="5"/>
-      <c r="E136" s="8" t="s">
-        <v>1318</v>
+      <c r="E136" s="7" t="s">
+        <v>1319</v>
       </c>
       <c r="F136" s="5"/>
       <c r="G136" s="5" t="s">
@@ -9402,7 +9403,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="140" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>139</v>
       </c>
@@ -9413,8 +9414,8 @@
         <v>925</v>
       </c>
       <c r="D140" s="5"/>
-      <c r="E140" s="8" t="s">
-        <v>1319</v>
+      <c r="E140" s="7" t="s">
+        <v>1320</v>
       </c>
       <c r="F140" s="5"/>
       <c r="G140" s="5" t="s">
@@ -9544,7 +9545,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="144" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>143</v>
       </c>
@@ -9555,8 +9556,8 @@
         <v>949</v>
       </c>
       <c r="D144" s="5"/>
-      <c r="E144" s="8" t="s">
-        <v>1320</v>
+      <c r="E144" s="7" t="s">
+        <v>1321</v>
       </c>
       <c r="F144" s="5"/>
       <c r="G144" s="5" t="s">
@@ -9686,7 +9687,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="148" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>147</v>
       </c>
@@ -9697,8 +9698,8 @@
         <v>973</v>
       </c>
       <c r="D148" s="5"/>
-      <c r="E148" s="8" t="s">
-        <v>1321</v>
+      <c r="E148" s="7" t="s">
+        <v>1322</v>
       </c>
       <c r="F148" s="5"/>
       <c r="G148" s="5" t="s">
@@ -9758,7 +9759,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="150" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>149</v>
       </c>
@@ -9769,8 +9770,8 @@
         <v>986</v>
       </c>
       <c r="D150" s="5"/>
-      <c r="E150" s="8" t="s">
-        <v>1322</v>
+      <c r="E150" s="7" t="s">
+        <v>1323</v>
       </c>
       <c r="F150" s="5"/>
       <c r="G150" s="5" t="s">
@@ -9830,7 +9831,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="152" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>151</v>
       </c>
@@ -9841,8 +9842,8 @@
         <v>999</v>
       </c>
       <c r="D152" s="5"/>
-      <c r="E152" s="8" t="s">
-        <v>1323</v>
+      <c r="E152" s="7" t="s">
+        <v>1324</v>
       </c>
       <c r="F152" s="5"/>
       <c r="G152" s="5" t="s">
@@ -9937,7 +9938,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="155" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -9948,8 +9949,8 @@
         <v>1017</v>
       </c>
       <c r="D155" s="6"/>
-      <c r="E155" s="9" t="s">
-        <v>1324</v>
+      <c r="E155" s="8" t="s">
+        <v>1325</v>
       </c>
       <c r="F155" s="6"/>
       <c r="G155" s="6" t="s">
@@ -10009,7 +10010,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="157" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -10020,8 +10021,8 @@
         <v>1030</v>
       </c>
       <c r="D157" s="6"/>
-      <c r="E157" s="9" t="s">
-        <v>1325</v>
+      <c r="E157" s="8" t="s">
+        <v>1326</v>
       </c>
       <c r="F157" s="6"/>
       <c r="G157" s="6" t="s">
@@ -10081,7 +10082,7 @@
         <v>1042</v>
       </c>
     </row>
-    <row r="159" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -10092,8 +10093,8 @@
         <v>1043</v>
       </c>
       <c r="D159" s="6"/>
-      <c r="E159" s="9" t="s">
-        <v>1326</v>
+      <c r="E159" s="8" t="s">
+        <v>1327</v>
       </c>
       <c r="F159" s="6"/>
       <c r="G159" s="6" t="s">
@@ -10223,7 +10224,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="163" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -10234,8 +10235,8 @@
         <v>1068</v>
       </c>
       <c r="D163" s="6"/>
-      <c r="E163" s="9" t="s">
-        <v>1327</v>
+      <c r="E163" s="8" t="s">
+        <v>1328</v>
       </c>
       <c r="F163" s="6"/>
       <c r="G163" s="6" t="s">
@@ -10365,7 +10366,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="167" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
         <v>166</v>
       </c>
@@ -10376,8 +10377,8 @@
         <v>1093</v>
       </c>
       <c r="D167" s="6"/>
-      <c r="E167" s="9" t="s">
-        <v>1328</v>
+      <c r="E167" s="8" t="s">
+        <v>1329</v>
       </c>
       <c r="F167" s="6"/>
       <c r="G167" s="6" t="s">
@@ -10472,7 +10473,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="170" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A170" s="4">
         <v>169</v>
       </c>
@@ -10483,8 +10484,8 @@
         <v>1112</v>
       </c>
       <c r="D170" s="5"/>
-      <c r="E170" s="8" t="s">
-        <v>1329</v>
+      <c r="E170" s="7" t="s">
+        <v>1330</v>
       </c>
       <c r="F170" s="5"/>
       <c r="G170" s="5" t="s">
@@ -10579,7 +10580,7 @@
         <v>1130</v>
       </c>
     </row>
-    <row r="173" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
         <v>172</v>
       </c>
@@ -10590,8 +10591,8 @@
         <v>1131</v>
       </c>
       <c r="D173" s="6"/>
-      <c r="E173" s="9" t="s">
-        <v>1330</v>
+      <c r="E173" s="8" t="s">
+        <v>1331</v>
       </c>
       <c r="F173" s="6"/>
       <c r="G173" s="6" t="s">
@@ -10721,7 +10722,7 @@
         <v>1151</v>
       </c>
     </row>
-    <row r="177" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" ht="135" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
         <v>176</v>
       </c>
@@ -10732,8 +10733,8 @@
         <v>1152</v>
       </c>
       <c r="D177" s="6"/>
-      <c r="E177" s="6" t="s">
-        <v>1331</v>
+      <c r="E177" s="8" t="s">
+        <v>1332</v>
       </c>
       <c r="F177" s="6"/>
       <c r="G177" s="6" t="s">
@@ -10909,8 +10910,8 @@
         <v>1183</v>
       </c>
       <c r="D182" s="5"/>
-      <c r="E182" s="5" t="s">
-        <v>1332</v>
+      <c r="E182" s="7" t="s">
+        <v>1333</v>
       </c>
       <c r="F182" s="5"/>
       <c r="G182" s="5" t="s">
@@ -11087,7 +11088,7 @@
       </c>
       <c r="D187" s="6"/>
       <c r="E187" s="6" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="F187" s="6"/>
       <c r="G187" s="6" t="s">
@@ -11252,7 +11253,7 @@
         <v>1243</v>
       </c>
     </row>
-    <row r="192" spans="1:13" ht="225" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" ht="210" x14ac:dyDescent="0.25">
       <c r="A192" s="4">
         <v>191</v>
       </c>
@@ -11264,7 +11265,7 @@
       </c>
       <c r="D192" s="5"/>
       <c r="E192" s="5" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="F192" s="5"/>
       <c r="G192" s="5" t="s">
@@ -11429,7 +11430,7 @@
         <v>1274</v>
       </c>
     </row>
-    <row r="197" spans="1:13" ht="225" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" ht="210" x14ac:dyDescent="0.25">
       <c r="A197" s="2">
         <v>196</v>
       </c>
@@ -11440,8 +11441,8 @@
         <v>1275</v>
       </c>
       <c r="D197" s="6"/>
-      <c r="E197" s="6" t="s">
-        <v>1335</v>
+      <c r="E197" s="8" t="s">
+        <v>1336</v>
       </c>
       <c r="F197" s="6"/>
       <c r="G197" s="6" t="s">
@@ -11616,22 +11617,26 @@
     <hyperlink ref="E7" r:id="rId6"/>
     <hyperlink ref="E64" r:id="rId7"/>
     <hyperlink ref="E67" r:id="rId8"/>
-    <hyperlink ref="E97" r:id="rId9"/>
-    <hyperlink ref="E100" r:id="rId10"/>
-    <hyperlink ref="E132" r:id="rId11"/>
-    <hyperlink ref="E136" r:id="rId12"/>
-    <hyperlink ref="E140" r:id="rId13"/>
-    <hyperlink ref="E144" r:id="rId14"/>
-    <hyperlink ref="E148" r:id="rId15"/>
-    <hyperlink ref="E150" r:id="rId16"/>
-    <hyperlink ref="E152" r:id="rId17"/>
-    <hyperlink ref="E155" r:id="rId18"/>
-    <hyperlink ref="E157" r:id="rId19"/>
-    <hyperlink ref="E159" r:id="rId20"/>
-    <hyperlink ref="E163" r:id="rId21"/>
-    <hyperlink ref="E167" r:id="rId22"/>
-    <hyperlink ref="E170" r:id="rId23"/>
-    <hyperlink ref="E173" r:id="rId24"/>
+    <hyperlink ref="E70" r:id="rId9"/>
+    <hyperlink ref="E97" r:id="rId10"/>
+    <hyperlink ref="E100" r:id="rId11"/>
+    <hyperlink ref="E132" r:id="rId12"/>
+    <hyperlink ref="E136" r:id="rId13"/>
+    <hyperlink ref="E140" r:id="rId14"/>
+    <hyperlink ref="E144" r:id="rId15"/>
+    <hyperlink ref="E148" r:id="rId16"/>
+    <hyperlink ref="E150" r:id="rId17"/>
+    <hyperlink ref="E152" r:id="rId18"/>
+    <hyperlink ref="E155" r:id="rId19"/>
+    <hyperlink ref="E157" r:id="rId20"/>
+    <hyperlink ref="E159" r:id="rId21"/>
+    <hyperlink ref="E163" r:id="rId22"/>
+    <hyperlink ref="E167" r:id="rId23"/>
+    <hyperlink ref="E170" r:id="rId24"/>
+    <hyperlink ref="E173" r:id="rId25"/>
+    <hyperlink ref="E177" r:id="rId26" display="https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458775/p7_176_1_TEST_1_2023_pnyl3i.png "/>
+    <hyperlink ref="E182" r:id="rId27" display="https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458776/p7_181_1_TEST_1_2023_rsoqhe.png"/>
+    <hyperlink ref="E197" r:id="rId28" display="https://res.cloudinary.com/dhmq07vzk/image/upload/v1782458781/p7_196_1_TEST_1_2023_cmfmak.png "/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>